<commit_message>
Apply Spanish numeric formats to OVE Excel files
</commit_message>
<xml_diff>
--- a/assets/data/bcv/excel/ove_bcv_pib_real_anual.xlsx
+++ b/assets/data/bcv/excel/ove_bcv_pib_real_anual.xlsx
@@ -17,7 +17,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="[$-es-ES]#,##0"/>
+    <numFmt numFmtId="165" formatCode="[$-es-ES]#,##0.00"/>
+  </numFmts>
   <fonts count="5">
     <font>
       <name val="Calibri"/>
@@ -69,7 +72,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -83,6 +86,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -114,6 +123,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -144,6 +156,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -507,10 +522,10 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="n">
+      <c r="A7" s="7" t="n">
         <v>2008</v>
       </c>
-      <c r="B7" s="4" t="n">
+      <c r="B7" s="8" t="n">
         <v>3.276408308619679</v>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -540,10 +555,10 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="n">
+      <c r="A8" s="7" t="n">
         <v>2009</v>
       </c>
-      <c r="B8" s="4" t="n">
+      <c r="B8" s="8" t="n">
         <v>-4.095858699654258</v>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -573,10 +588,10 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="n">
+      <c r="A9" s="7" t="n">
         <v>2010</v>
       </c>
-      <c r="B9" s="4" t="n">
+      <c r="B9" s="8" t="n">
         <v>-0.6620080132279327</v>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -606,10 +621,10 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="n">
+      <c r="A10" s="7" t="n">
         <v>2011</v>
       </c>
-      <c r="B10" s="4" t="n">
+      <c r="B10" s="8" t="n">
         <v>2.728942883695225</v>
       </c>
       <c r="C10" s="4" t="inlineStr">
@@ -639,10 +654,10 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="n">
+      <c r="A11" s="7" t="n">
         <v>2012</v>
       </c>
-      <c r="B11" s="4" t="n">
+      <c r="B11" s="8" t="n">
         <v>4.243300030305591</v>
       </c>
       <c r="C11" s="4" t="inlineStr">
@@ -672,10 +687,10 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="n">
+      <c r="A12" s="7" t="n">
         <v>2013</v>
       </c>
-      <c r="B12" s="4" t="n">
+      <c r="B12" s="8" t="n">
         <v>0.07771331367443679</v>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -705,10 +720,10 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="n">
+      <c r="A13" s="7" t="n">
         <v>2014</v>
       </c>
-      <c r="B13" s="4" t="n">
+      <c r="B13" s="8" t="n">
         <v>-2.305807182523338</v>
       </c>
       <c r="C13" s="4" t="inlineStr">
@@ -738,10 +753,10 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="n">
+      <c r="A14" s="7" t="n">
         <v>2015</v>
       </c>
-      <c r="B14" s="4" t="n">
+      <c r="B14" s="8" t="n">
         <v>-3.868720967947553</v>
       </c>
       <c r="C14" s="4" t="inlineStr">
@@ -771,10 +786,10 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="n">
+      <c r="A15" s="7" t="n">
         <v>2016</v>
       </c>
-      <c r="B15" s="4" t="n">
+      <c r="B15" s="8" t="n">
         <v>-16.97801742690727</v>
       </c>
       <c r="C15" s="4" t="inlineStr">
@@ -804,10 +819,10 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="n">
+      <c r="A16" s="7" t="n">
         <v>2017</v>
       </c>
-      <c r="B16" s="4" t="n">
+      <c r="B16" s="8" t="n">
         <v>-14.42010721738242</v>
       </c>
       <c r="C16" s="4" t="inlineStr">
@@ -837,10 +852,10 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="n">
+      <c r="A17" s="7" t="n">
         <v>2018</v>
       </c>
-      <c r="B17" s="4" t="n">
+      <c r="B17" s="8" t="n">
         <v>-21.39586857963141</v>
       </c>
       <c r="C17" s="4" t="inlineStr">
@@ -870,10 +885,10 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="4" t="n">
+      <c r="A18" s="7" t="n">
         <v>2019</v>
       </c>
-      <c r="B18" s="4" t="n">
+      <c r="B18" s="8" t="n">
         <v>-28.99145829523422</v>
       </c>
       <c r="C18" s="4" t="inlineStr">
@@ -903,10 +918,10 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="n">
+      <c r="A19" s="7" t="n">
         <v>2020</v>
       </c>
-      <c r="B19" s="4" t="n">
+      <c r="B19" s="8" t="n">
         <v>-33.20381272402878</v>
       </c>
       <c r="C19" s="4" t="inlineStr">
@@ -936,10 +951,10 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="n">
+      <c r="A20" s="7" t="n">
         <v>2021</v>
       </c>
-      <c r="B20" s="4" t="n">
+      <c r="B20" s="8" t="n">
         <v>1.111016250264043</v>
       </c>
       <c r="C20" s="4" t="inlineStr">
@@ -969,10 +984,10 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="n">
+      <c r="A21" s="7" t="n">
         <v>2022</v>
       </c>
-      <c r="B21" s="4" t="n">
+      <c r="B21" s="8" t="n">
         <v>14.91768022765017</v>
       </c>
       <c r="C21" s="4" t="inlineStr">
@@ -1002,10 +1017,10 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="4" t="n">
+      <c r="A22" s="7" t="n">
         <v>2023</v>
       </c>
-      <c r="B22" s="4" t="n">
+      <c r="B22" s="8" t="n">
         <v>5.143618581513593</v>
       </c>
       <c r="C22" s="4" t="inlineStr">
@@ -1035,10 +1050,10 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="4" t="n">
+      <c r="A23" s="7" t="n">
         <v>2024</v>
       </c>
-      <c r="B23" s="4" t="n">
+      <c r="B23" s="8" t="n">
         <v>9.025539143402</v>
       </c>
       <c r="C23" s="4" t="inlineStr">
@@ -1068,10 +1083,10 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="4" t="n">
+      <c r="A24" s="7" t="n">
         <v>2025</v>
       </c>
-      <c r="B24" s="4" t="n">
+      <c r="B24" s="8" t="n">
         <v>8.944487326024571</v>
       </c>
       <c r="C24" s="4" t="inlineStr">
@@ -1238,7 +1253,7 @@
           <t>first_year</t>
         </is>
       </c>
-      <c r="B14" s="4" t="n">
+      <c r="B14" s="7" t="n">
         <v>2008</v>
       </c>
     </row>
@@ -1248,7 +1263,7 @@
           <t>last_year</t>
         </is>
       </c>
-      <c r="B15" s="4" t="n">
+      <c r="B15" s="7" t="n">
         <v>2025</v>
       </c>
     </row>
@@ -1258,7 +1273,7 @@
           <t>records</t>
         </is>
       </c>
-      <c r="B16" s="4" t="n">
+      <c r="B16" s="7" t="n">
         <v>18</v>
       </c>
     </row>

</xml_diff>